<commit_message>
CDM/ontology: Building, PolicyTransaction and ClaimFinancial are related objects, not subclasses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PQwjCCpYmPMPxiBbaix3n8
</commit_message>
<xml_diff>
--- a/website/downloads/SI2_Commercial_CDM.xlsx
+++ b/website/downloads/SI2_Commercial_CDM.xlsx
@@ -18547,11 +18547,7 @@
           <t>Policy transaction</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Policy</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>New business, endorsement, cancellation, reinstatement, renewal or audit.</t>
@@ -18597,11 +18593,7 @@
           <t>Building</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>A structure at a location (Commercial Property).</t>
@@ -18789,11 +18781,7 @@
           <t>Claim financial transaction</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Claim</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Payment, recovery or reserve change.</t>

</xml_diff>